<commit_message>
cambios en el formato
cambios en el formato
</commit_message>
<xml_diff>
--- a/FORMATO PARA CARGAR LAS NOTAS.xlsx
+++ b/FORMATO PARA CARGAR LAS NOTAS.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F6F5AF-04CA-4DEF-AACF-7EE06C05DAC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A63DE1-38D2-4B40-8D98-C568439E048D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
   <si>
     <t>UNIDAD EDUCATIVA EMILIANO HINOSTROZA</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t xml:space="preserve">EDUCACION INICIAL </t>
+  </si>
+  <si>
+    <t>EVALUACIÓN COMPORTAMENTAL</t>
   </si>
 </sst>
 </file>
@@ -692,6 +695,7 @@
     <col min="5" max="12" width="30" customWidth="1"/>
     <col min="13" max="13" width="49.88671875" customWidth="1"/>
     <col min="14" max="17" width="30" customWidth="1"/>
+    <col min="18" max="18" width="34.109375" customWidth="1"/>
     <col min="27" max="27" width="0" hidden="1" customWidth="1"/>
     <col min="28" max="28" width="39.21875" hidden="1" customWidth="1"/>
     <col min="29" max="29" width="33.21875" hidden="1" customWidth="1"/>
@@ -913,6 +917,9 @@
       </c>
       <c r="Q9" s="2" t="s">
         <v>16</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="AB9" t="s">
         <v>72</v>
@@ -942,6 +949,7 @@
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
       <c r="AC10" t="s">
         <v>53</v>
       </c>
@@ -967,6 +975,7 @@
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
       <c r="AC11" t="s">
         <v>54</v>
       </c>
@@ -992,6 +1001,7 @@
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
+      <c r="R12" s="3"/>
       <c r="AC12" t="s">
         <v>55</v>
       </c>
@@ -1017,6 +1027,7 @@
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
+      <c r="R13" s="3"/>
       <c r="AC13" t="s">
         <v>56</v>
       </c>
@@ -1042,6 +1053,7 @@
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
+      <c r="R14" s="3"/>
       <c r="AC14" t="s">
         <v>57</v>
       </c>
@@ -1067,6 +1079,7 @@
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
+      <c r="R15" s="3"/>
       <c r="AC15" t="s">
         <v>58</v>
       </c>
@@ -1089,6 +1102,7 @@
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
+      <c r="R16" s="3"/>
       <c r="AC16" t="s">
         <v>59</v>
       </c>

</xml_diff>